<commit_message>
Added header, change paragraphs
</commit_message>
<xml_diff>
--- a/Mariana_Garcia_gantt chart.xlsx
+++ b/Mariana_Garcia_gantt chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria\Desktop\DATA ANALYTICS\LEVEL 8\Business Strategy\CCT_Capstone_Online_Shoppers\Figures\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria\Documents\GitHub\Capstone-Project---2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78638508-F119-4BDA-843B-46DF05200997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF8CFA69-1A18-41DF-A150-59C8884536EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E55E00BB-72E4-4B08-A6C8-86E5C9753136}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E55E00BB-72E4-4B08-A6C8-86E5C9753136}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="39">
   <si>
     <t>Dataset exploration and analysis</t>
   </si>
@@ -99,9 +99,6 @@
     <t>2nd Semestre 2027</t>
   </si>
   <si>
-    <t>The project will be completed over two semesters: September–December 2026 and January–May 2027. Semester 1 will focus on research, data understanding and preliminary analysis. Semester 2 will focus on predictive modelling, evaluation, visualisation and the final report.</t>
-  </si>
-  <si>
     <t>Key milestones</t>
   </si>
   <si>
@@ -157,6 +154,12 @@
   </si>
   <si>
     <t>Final submission</t>
+  </si>
+  <si>
+    <t>The project will be completed over two semesters: September–December 2026 and January–May 2027.</t>
+  </si>
+  <si>
+    <t>Data preparation completed</t>
   </si>
 </sst>
 </file>
@@ -167,7 +170,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
     <numFmt numFmtId="165" formatCode="m/d/yy;@"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -191,14 +194,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -213,13 +208,36 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Cambria"/>
-      <family val="1"/>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -368,71 +386,29 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="17" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="17" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -442,8 +418,45 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="17" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -790,105 +803,105 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A948B434-6211-4343-A41C-5E6C75935B20}">
-  <dimension ref="A1:Q27"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.36328125" customWidth="1"/>
-    <col min="2" max="2" width="11.453125" customWidth="1"/>
-    <col min="3" max="3" width="11.6328125" customWidth="1"/>
+    <col min="1" max="1" width="49" customWidth="1"/>
+    <col min="2" max="2" width="22.54296875" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="8.81640625" customWidth="1"/>
     <col min="15" max="15" width="18" customWidth="1"/>
     <col min="16" max="16" width="20" customWidth="1"/>
     <col min="17" max="17" width="12.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="40.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="O1" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
-      <c r="L1" s="31"/>
-      <c r="O1" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="P1" s="21" t="s">
+      <c r="P1" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="Q1" s="21" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="27" t="s">
+    </row>
+    <row r="2" spans="1:17" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="J2" s="27"/>
-      <c r="K2" s="27"/>
-      <c r="L2" s="27"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
       <c r="O2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="P2" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>27</v>
       </c>
       <c r="Q2" s="3">
         <v>46320</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="22" t="s">
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13"/>
+      <c r="K3" s="13"/>
+      <c r="L3" s="13"/>
       <c r="O3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="P3" s="20" t="s">
-        <v>34</v>
+        <v>29</v>
+      </c>
+      <c r="P3" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="Q3" s="3">
         <v>46410</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A4" s="24"/>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
+      <c r="A4" s="28"/>
+      <c r="B4" s="29"/>
+      <c r="C4" s="29"/>
       <c r="D4" s="2">
         <v>46266</v>
       </c>
@@ -919,23 +932,23 @@
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="3">
         <v>46476</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A5" s="12" t="s">
+    <row r="5" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A5" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="18">
+      <c r="B5" s="24">
         <v>46293</v>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="24">
         <v>46300</v>
       </c>
       <c r="D5" s="4"/>
@@ -948,23 +961,23 @@
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
       <c r="O5" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P5" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q5" s="3">
         <v>46507</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A6" s="12" t="s">
+    <row r="6" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A6" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="24">
         <v>46300</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="24">
         <v>46304</v>
       </c>
       <c r="D6" s="4"/>
@@ -977,23 +990,23 @@
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
       <c r="O6" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="Q6" s="3">
         <v>46537</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A7" s="12" t="s">
+    <row r="7" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A7" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="24">
         <v>46304</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="24">
         <v>46307</v>
       </c>
       <c r="D7" s="4"/>
@@ -1006,14 +1019,14 @@
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A8" s="12" t="s">
+    <row r="8" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A8" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="24">
         <v>46307</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="24">
         <v>46320</v>
       </c>
       <c r="D8" s="4"/>
@@ -1026,19 +1039,19 @@
       <c r="K8" s="5"/>
       <c r="L8" s="5"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A9" s="13" t="s">
+    <row r="9" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A9" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="24">
+        <v>46320</v>
+      </c>
+      <c r="C9" s="24">
+        <v>46320</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="10" t="s">
         <v>20</v>
-      </c>
-      <c r="B9" s="18">
-        <v>46320</v>
-      </c>
-      <c r="C9" s="18">
-        <v>46320</v>
-      </c>
-      <c r="D9" s="3"/>
-      <c r="E9" s="11" t="s">
-        <v>21</v>
       </c>
       <c r="F9" s="5"/>
       <c r="G9" s="5"/>
@@ -1048,14 +1061,14 @@
       <c r="K9" s="5"/>
       <c r="L9" s="5"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A10" s="14" t="s">
+    <row r="10" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A10" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="24">
         <v>46320</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="24">
         <v>46350</v>
       </c>
       <c r="D10" s="3"/>
@@ -1068,14 +1081,14 @@
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A11" s="14" t="s">
+    <row r="11" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A11" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="24">
         <v>46350</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="24">
         <v>46380</v>
       </c>
       <c r="D11" s="3"/>
@@ -1088,14 +1101,14 @@
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A12" s="14" t="s">
+    <row r="12" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A12" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="18">
+      <c r="B12" s="24">
         <v>46380</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="24">
         <v>46410</v>
       </c>
       <c r="D12" s="3"/>
@@ -1108,36 +1121,36 @@
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A13" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B13" s="18">
+    <row r="13" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A13" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="24">
         <v>46410</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="24">
         <v>46410</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="5"/>
       <c r="F13" s="7"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="11" t="s">
-        <v>21</v>
+      <c r="H13" s="10" t="s">
+        <v>20</v>
       </c>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A14" s="15" t="s">
+    <row r="14" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A14" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="18">
+      <c r="B14" s="24">
         <v>46411</v>
       </c>
-      <c r="C14" s="18">
+      <c r="C14" s="24">
         <v>46476</v>
       </c>
       <c r="D14" s="3"/>
@@ -1150,14 +1163,14 @@
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="18">
+    <row r="15" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A15" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="24">
         <v>46476</v>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="24">
         <v>46476</v>
       </c>
       <c r="D15" s="3"/>
@@ -1166,20 +1179,20 @@
       <c r="G15" s="5"/>
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
-      <c r="J15" s="11" t="s">
-        <v>21</v>
+      <c r="J15" s="10" t="s">
+        <v>20</v>
       </c>
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A16" s="15" t="s">
+    <row r="16" spans="1:17" ht="21" x14ac:dyDescent="0.35">
+      <c r="A16" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="24">
         <v>46476</v>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="24">
         <v>46507</v>
       </c>
       <c r="D16" s="3"/>
@@ -1192,14 +1205,14 @@
       <c r="K16" s="8"/>
       <c r="L16" s="5"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A17" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B17" s="18">
+    <row r="17" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="A17" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="24">
         <v>46507</v>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="24">
         <v>46507</v>
       </c>
       <c r="D17" s="3"/>
@@ -1209,19 +1222,19 @@
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
-      <c r="K17" s="11" t="s">
-        <v>21</v>
+      <c r="K17" s="10" t="s">
+        <v>20</v>
       </c>
       <c r="L17" s="5"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A18" s="17" t="s">
+    <row r="18" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="A18" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="18">
+      <c r="B18" s="24">
         <v>46507</v>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="24">
         <v>46517</v>
       </c>
       <c r="D18" s="3"/>
@@ -1234,14 +1247,14 @@
       <c r="K18" s="9"/>
       <c r="L18" s="9"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A19" s="17" t="s">
+    <row r="19" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="A19" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="24">
         <v>46507</v>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="24">
         <v>46517</v>
       </c>
       <c r="D19" s="3"/>
@@ -1254,14 +1267,14 @@
       <c r="K19" s="9"/>
       <c r="L19" s="9"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A20" s="17" t="s">
+    <row r="20" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+      <c r="A20" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="18">
+      <c r="B20" s="24">
         <v>46517</v>
       </c>
-      <c r="C20" s="18">
+      <c r="C20" s="24">
         <v>46537</v>
       </c>
       <c r="D20" s="3"/>
@@ -1274,14 +1287,14 @@
       <c r="K20" s="5"/>
       <c r="L20" s="9"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A21" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B21" s="3">
+    <row r="21" spans="1:12" ht="21" x14ac:dyDescent="0.5">
+      <c r="A21" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="25">
         <v>46537</v>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="25">
         <v>46537</v>
       </c>
       <c r="D21" s="3"/>
@@ -1292,21 +1305,78 @@
       <c r="I21" s="5"/>
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
-      <c r="L21" s="11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A23" s="10"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
+      <c r="L21" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A23" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" s="26" t="s">
+        <v>28</v>
+      </c>
       <c r="D23" s="1"/>
     </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A24" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="3">
+        <v>46320</v>
+      </c>
+    </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A25" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="3">
+        <v>46410</v>
+      </c>
       <c r="D25" s="1"/>
     </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A26" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="3">
+        <v>46476</v>
+      </c>
+    </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A27" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="3">
+        <v>46507</v>
+      </c>
       <c r="D27" s="1"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A28" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C28" s="3">
+        <v>46537</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1319,6 +1389,7 @@
     <mergeCell ref="D3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1333,22 +1404,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="B1" s="21" t="s">
+      <c r="A1" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="12" t="s">
         <v>28</v>
-      </c>
-      <c r="C1" s="21" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>27</v>
       </c>
       <c r="C2" s="3">
         <v>46320</v>
@@ -1356,10 +1427,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>34</v>
+        <v>29</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="C3" s="3">
         <v>46410</v>
@@ -1367,10 +1438,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" s="3">
         <v>46476</v>
@@ -1378,10 +1449,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" s="3">
         <v>46507</v>
@@ -1389,17 +1460,17 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" s="3">
         <v>46537</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Changed Gantt Chart dates
</commit_message>
<xml_diff>
--- a/Mariana_Garcia_gantt chart.xlsx
+++ b/Mariana_Garcia_gantt chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maria\Documents\GitHub\Capstone-Project---2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF8CFA69-1A18-41DF-A150-59C8884536EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65DC51D7-95FA-4128-A6D3-2CE328D54A84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E55E00BB-72E4-4B08-A6C8-86E5C9753136}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="39">
   <si>
     <t>Dataset exploration and analysis</t>
   </si>
@@ -156,10 +156,10 @@
     <t>Final submission</t>
   </si>
   <si>
-    <t>The project will be completed over two semesters: September–December 2026 and January–May 2027.</t>
-  </si>
-  <si>
     <t>Data preparation completed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proposal submitted </t>
   </si>
 </sst>
 </file>
@@ -305,7 +305,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -376,6 +376,83 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -386,7 +463,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="17" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -406,9 +483,43 @@
     </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="17" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -418,44 +529,30 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="17" fontId="4" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="17" fontId="4" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -803,33 +900,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A948B434-6211-4343-A41C-5E6C75935B20}">
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="49" customWidth="1"/>
     <col min="2" max="2" width="22.54296875" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="8.81640625" customWidth="1"/>
+    <col min="13" max="13" width="8.7265625" style="31"/>
     <col min="15" max="15" width="18" customWidth="1"/>
     <col min="16" max="16" width="20" customWidth="1"/>
     <col min="17" max="17" width="12.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="21" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
+      <c r="A1" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="37"/>
       <c r="O1" s="12" t="s">
         <v>18</v>
       </c>
@@ -840,21 +938,19 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="30" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
+    <row r="2" spans="1:17" ht="23.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="38"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
+      <c r="K2" s="39"/>
+      <c r="L2" s="40"/>
       <c r="O2" s="5" t="s">
         <v>25</v>
       </c>
@@ -866,28 +962,28 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="14" t="s">
+      <c r="D3" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="13" t="s">
+      <c r="E3" s="27"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
       <c r="O3" s="5" t="s">
         <v>29</v>
       </c>
@@ -899,9 +995,9 @@
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A4" s="28"/>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
       <c r="D4" s="2">
         <v>46266</v>
       </c>
@@ -929,7 +1025,7 @@
       <c r="L4" s="2">
         <v>46508</v>
       </c>
-      <c r="M4" s="1"/>
+      <c r="M4" s="34"/>
       <c r="N4" s="1"/>
       <c r="O4" s="5" t="s">
         <v>30</v>
@@ -942,13 +1038,13 @@
       </c>
     </row>
     <row r="5" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="24">
+      <c r="B5" s="19">
         <v>46293</v>
       </c>
-      <c r="C5" s="24">
+      <c r="C5" s="19">
         <v>46300</v>
       </c>
       <c r="D5" s="4"/>
@@ -971,13 +1067,13 @@
       </c>
     </row>
     <row r="6" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="24">
+      <c r="B6" s="19">
         <v>46300</v>
       </c>
-      <c r="C6" s="24">
+      <c r="C6" s="19">
         <v>46304</v>
       </c>
       <c r="D6" s="4"/>
@@ -1000,13 +1096,13 @@
       </c>
     </row>
     <row r="7" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="24">
+      <c r="B7" s="19">
         <v>46304</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="19">
         <v>46307</v>
       </c>
       <c r="D7" s="4"/>
@@ -1020,13 +1116,13 @@
       <c r="L7" s="5"/>
     </row>
     <row r="8" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="24">
+      <c r="B8" s="19">
         <v>46307</v>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="19">
         <v>46320</v>
       </c>
       <c r="D8" s="4"/>
@@ -1040,13 +1136,13 @@
       <c r="L8" s="5"/>
     </row>
     <row r="9" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="24">
+      <c r="B9" s="19">
         <v>46320</v>
       </c>
-      <c r="C9" s="24">
+      <c r="C9" s="19">
         <v>46320</v>
       </c>
       <c r="D9" s="3"/>
@@ -1062,13 +1158,13 @@
       <c r="L9" s="5"/>
     </row>
     <row r="10" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="24">
+      <c r="B10" s="19">
         <v>46320</v>
       </c>
-      <c r="C10" s="24">
+      <c r="C10" s="19">
         <v>46350</v>
       </c>
       <c r="D10" s="3"/>
@@ -1082,13 +1178,13 @@
       <c r="L10" s="5"/>
     </row>
     <row r="11" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="24">
+      <c r="B11" s="19">
         <v>46350</v>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="19">
         <v>46380</v>
       </c>
       <c r="D11" s="3"/>
@@ -1102,13 +1198,13 @@
       <c r="L11" s="5"/>
     </row>
     <row r="12" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A12" s="19" t="s">
+      <c r="A12" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="24">
+      <c r="B12" s="19">
         <v>46380</v>
       </c>
-      <c r="C12" s="24">
+      <c r="C12" s="19">
         <v>46410</v>
       </c>
       <c r="D12" s="3"/>
@@ -1122,13 +1218,13 @@
       <c r="L12" s="5"/>
     </row>
     <row r="13" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A13" s="18" t="s">
+      <c r="A13" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="24">
+      <c r="B13" s="19">
         <v>46410</v>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="19">
         <v>46410</v>
       </c>
       <c r="D13" s="3"/>
@@ -1144,13 +1240,13 @@
       <c r="L13" s="5"/>
     </row>
     <row r="14" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="24">
+      <c r="B14" s="19">
         <v>46411</v>
       </c>
-      <c r="C14" s="24">
+      <c r="C14" s="19">
         <v>46476</v>
       </c>
       <c r="D14" s="3"/>
@@ -1164,13 +1260,13 @@
       <c r="L14" s="5"/>
     </row>
     <row r="15" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="24">
+      <c r="B15" s="19">
         <v>46476</v>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="19">
         <v>46476</v>
       </c>
       <c r="D15" s="3"/>
@@ -1186,13 +1282,13 @@
       <c r="L15" s="5"/>
     </row>
     <row r="16" spans="1:17" ht="21" x14ac:dyDescent="0.35">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B16" s="24">
-        <v>46476</v>
-      </c>
-      <c r="C16" s="24">
+      <c r="B16" s="19">
+        <v>46477</v>
+      </c>
+      <c r="C16" s="19">
         <v>46507</v>
       </c>
       <c r="D16" s="3"/>
@@ -1206,13 +1302,13 @@
       <c r="L16" s="5"/>
     </row>
     <row r="17" spans="1:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="24">
+      <c r="B17" s="19">
         <v>46507</v>
       </c>
-      <c r="C17" s="24">
+      <c r="C17" s="19">
         <v>46507</v>
       </c>
       <c r="D17" s="3"/>
@@ -1228,13 +1324,13 @@
       <c r="L17" s="5"/>
     </row>
     <row r="18" spans="1:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="24">
+      <c r="B18" s="19">
         <v>46507</v>
       </c>
-      <c r="C18" s="24">
+      <c r="C18" s="19">
         <v>46517</v>
       </c>
       <c r="D18" s="3"/>
@@ -1248,13 +1344,13 @@
       <c r="L18" s="9"/>
     </row>
     <row r="19" spans="1:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="24">
+      <c r="B19" s="19">
         <v>46507</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="19">
         <v>46517</v>
       </c>
       <c r="D19" s="3"/>
@@ -1268,13 +1364,13 @@
       <c r="L19" s="9"/>
     </row>
     <row r="20" spans="1:12" ht="21" x14ac:dyDescent="0.35">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="24">
+      <c r="B20" s="19">
         <v>46517</v>
       </c>
-      <c r="C20" s="24">
+      <c r="C20" s="19">
         <v>46537</v>
       </c>
       <c r="D20" s="3"/>
@@ -1288,13 +1384,13 @@
       <c r="L20" s="9"/>
     </row>
     <row r="21" spans="1:12" ht="21" x14ac:dyDescent="0.5">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="25">
+      <c r="B21" s="20">
         <v>46537</v>
       </c>
-      <c r="C21" s="25">
+      <c r="C21" s="20">
         <v>46537</v>
       </c>
       <c r="D21" s="3"/>
@@ -1309,40 +1405,76 @@
         <v>20</v>
       </c>
     </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="31"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="31"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
+      <c r="L22" s="31"/>
+    </row>
     <row r="23" spans="1:12" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A23" s="26" t="s">
+      <c r="A23" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="B23" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="26" t="s">
+      <c r="C23" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="D23" s="1"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="30"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="30"/>
+      <c r="H23" s="30"/>
+      <c r="I23" s="30"/>
+      <c r="J23" s="30"/>
+      <c r="K23" s="30"/>
+      <c r="L23" s="30"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C24" s="3">
+        <v>38</v>
+      </c>
+      <c r="C24" s="33">
         <v>46320</v>
       </c>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+      <c r="H24" s="30"/>
+      <c r="I24" s="30"/>
+      <c r="J24" s="30"/>
+      <c r="K24" s="30"/>
+      <c r="L24" s="30"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C25" s="3">
+        <v>37</v>
+      </c>
+      <c r="C25" s="33">
         <v>46410</v>
       </c>
-      <c r="D25" s="1"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="30"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="30"/>
+      <c r="H25" s="30"/>
+      <c r="I25" s="30"/>
+      <c r="J25" s="30"/>
+      <c r="K25" s="30"/>
+      <c r="L25" s="30"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" s="5" t="s">
@@ -1351,9 +1483,18 @@
       <c r="B26" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C26" s="3">
+      <c r="C26" s="33">
         <v>46476</v>
       </c>
+      <c r="D26" s="30"/>
+      <c r="E26" s="30"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="30"/>
+      <c r="H26" s="30"/>
+      <c r="I26" s="30"/>
+      <c r="J26" s="30"/>
+      <c r="K26" s="30"/>
+      <c r="L26" s="30"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" s="5" t="s">
@@ -1362,10 +1503,18 @@
       <c r="B27" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C27" s="3">
+      <c r="C27" s="33">
         <v>46507</v>
       </c>
-      <c r="D27" s="1"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="30"/>
+      <c r="I27" s="30"/>
+      <c r="J27" s="30"/>
+      <c r="K27" s="30"/>
+      <c r="L27" s="30"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A28" s="5" t="s">
@@ -1374,19 +1523,60 @@
       <c r="B28" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C28" s="3">
+      <c r="C28" s="33">
         <v>46537</v>
       </c>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="31"/>
+      <c r="J29" s="31"/>
+      <c r="K29" s="31"/>
+      <c r="L29" s="31"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="31"/>
+      <c r="J30" s="31"/>
+      <c r="K30" s="31"/>
+      <c r="L30" s="31"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="D31" s="31"/>
+      <c r="E31" s="31"/>
+      <c r="F31" s="31"/>
+      <c r="G31" s="31"/>
+      <c r="H31" s="31"/>
+      <c r="I31" s="31"/>
+      <c r="J31" s="31"/>
+      <c r="K31" s="31"/>
+      <c r="L31" s="31"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A1:L1"/>
+  <mergeCells count="6">
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
-    <mergeCell ref="A2:L2"/>
     <mergeCell ref="D3:G3"/>
+    <mergeCell ref="A1:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>